<commit_message>
Reword the dairy and brewery case studies as model documentation
The six case studies no longer address students ("you design", "check
your own", "handout", rs/qt headings): they gain their authors and
affiliation and a scope paragraph that ties each to its database model
and sources. The data workbooks lose their two course sentences, and the
Lua headers name the workbooks as they are in Documents.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/3-IndustrialProcesses/FoodAndBeverage/Brewery/Documents/BreweryBiog_V1_rs_qt.xlsx
+++ b/3-IndustrialProcesses/FoodAndBeverage/Brewery/Documents/BreweryBiog_V1_rs_qt.xlsx
@@ -75,7 +75,7 @@
     <t xml:space="preserve">dTmin/2 = 5 K for liquid streams and 2 K for wort evaporation and vapour condensation; isothermal streams have a 0.1 K span.</t>
   </si>
   <si>
-    <t xml:space="preserve">Corrections to the source (pasteurisation at 70 C, whirlpool make-up water, dilution water) are listed in the handout, section Data basis.</t>
+    <t xml:space="preserve">Corrections to the source (pasteurisation at 70 C, whirlpool make-up water, dilution water) are listed in the case study, section Data basis.</t>
   </si>
   <si>
     <t xml:space="preserve">Utilities (steam, hot water, glycol-water, ammonia refrigeration, cooling water) are not part of the process data.</t>
@@ -735,7 +735,7 @@
     <t xml:space="preserve">Reference targets for the 29 streams of the qt sheet</t>
   </si>
   <si>
-    <t xml:space="preserve">Problem-table results with the dTmin/2 of each stream, given as values to check your own calculation.</t>
+    <t xml:space="preserve">Problem-table results with the dTmin/2 of each stream.</t>
   </si>
   <si>
     <t xml:space="preserve">Quantity</t>

</xml_diff>